<commit_message>
Add Column Gatepass, Add Download button Storagebin List
</commit_message>
<xml_diff>
--- a/SEMB_ERP/wwwroot/template/Template_Upload_Material.xlsx
+++ b/SEMB_ERP/wwwroot/template/Template_Upload_Material.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SESA546923\Documents\GitHub\SEMB_ERP\SEMB_ERP\wwwroot\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sesa732369\Documents\GitHub\SEMB_ERP\SEMB_ERP\wwwroot\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF6E36C8-6B46-428A-80AF-2F4228AC54B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D54C4B6-A394-4C1C-B594-6366B81F2A51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{610016C1-593C-4B28-8FE2-E321024077D0}"/>
+    <workbookView xWindow="3855" yWindow="3855" windowWidth="21600" windowHeight="12645" xr2:uid="{610016C1-593C-4B28-8FE2-E321024077D0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="34">
   <si>
     <t>Material Type</t>
   </si>
@@ -268,6 +268,9 @@
   </si>
   <si>
     <t>RM</t>
+  </si>
+  <si>
+    <t>Gatepass</t>
   </si>
 </sst>
 </file>
@@ -341,9 +344,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -381,7 +384,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -487,7 +490,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -629,7 +632,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -637,27 +640,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AAC486F-9B95-4840-90FB-639F5A25D6B8}">
-  <dimension ref="A1:O3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:P3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.5546875" customWidth="1"/>
-    <col min="12" max="12" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.5546875" customWidth="1"/>
-    <col min="14" max="14" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.6640625" customWidth="1"/>
+    <col min="11" max="11" width="10.5703125" customWidth="1"/>
+    <col min="12" max="12" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.5703125" customWidth="1"/>
+    <col min="14" max="14" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -703,8 +706,11 @@
       <c r="O1" t="s">
         <v>3</v>
       </c>
+      <c r="P1" t="s">
+        <v>33</v>
+      </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>32</v>
       </c>
@@ -750,8 +756,11 @@
       <c r="O2" t="s">
         <v>3</v>
       </c>
+      <c r="P2" t="s">
+        <v>33</v>
+      </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -796,6 +805,9 @@
       </c>
       <c r="O3" t="s">
         <v>3</v>
+      </c>
+      <c r="P3" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -833,13 +845,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C8463B8-D4B7-4837-A0E8-8C134D18F8A6}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -850,7 +862,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>32</v>
       </c>
@@ -861,7 +873,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -872,7 +884,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -886,4 +898,10 @@
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;6&amp;K626469 Public</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{23507802-f8e4-4e38-829c-ac8ea9b241e4}" enabled="1" method="Privileged" siteId="{6e51e1ad-c54b-4b39-b598-0ffe9ae68fef}" contentBits="2" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>